<commit_message>
feat: Add Gemini evaluator and implement detailed test reporting dashboard with new report files.
</commit_message>
<xml_diff>
--- a/assets/xlsx/testing.xlsx
+++ b/assets/xlsx/testing.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GITHUB\migrasiplaywright12345\assets\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GITHUB\automationtestingjudges\assets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1891C57-40E2-4AAA-A14D-4F4E7EFE18A8}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C877B567-2A02-47EC-9375-759DAEFD79BA}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,13 +42,13 @@
     <t>Apa itu asuransi jiwa</t>
   </si>
   <si>
-    <t>Jenis asuransi ini memberikan perlindungan finansial terhadap risiko kehidupan dan kematian pemegang polis.</t>
-  </si>
-  <si>
     <t>Apa itu asuransi kesehatan</t>
   </si>
   <si>
     <t>Asuransi kesehatan merupakan jenis asuransi yang memberikan perlindungan finansial ketika mengalami masalah kesehatan.</t>
+  </si>
+  <si>
+    <t>HIDUP JOKOWI!!</t>
   </si>
 </sst>
 </file>
@@ -521,7 +521,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -529,13 +529,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>